<commit_message>
update(data): perbarui data sekolah Book2.xlsx BauBau (penambahan kecamatan LEA-LEA)
</commit_message>
<xml_diff>
--- a/public/Book2.xlsx
+++ b/public/Book2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Rupa-Rupa\EduEvent\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{12EBD738-9A91-4872-8FB5-1B3D2ACEB12F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DB56EC26-1AAB-4B86-9CF0-2B008C6C6CF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{778D8361-FF95-495E-9D13-953602A5D773}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="80">
   <si>
     <t>Nama Sekolah</t>
   </si>
@@ -252,6 +252,30 @@
   </si>
   <si>
     <t>BUNGI</t>
+  </si>
+  <si>
+    <t>SD NEGERI 1 BATARAGURU</t>
+  </si>
+  <si>
+    <t>SD NEGERI KALIALIA</t>
+  </si>
+  <si>
+    <t>SD NEGERI 3 LOWU-LOWU</t>
+  </si>
+  <si>
+    <t>SD NEGERI 2 LOWU-LOWU</t>
+  </si>
+  <si>
+    <t>SD NEGERI 1 LOWU-LOWU</t>
+  </si>
+  <si>
+    <t>SD NEGERI KECIL KOLAGANA</t>
+  </si>
+  <si>
+    <t>SD NEGERI KECIL WAMEMBE</t>
+  </si>
+  <si>
+    <t>LEA-LEA</t>
   </si>
 </sst>
 </file>
@@ -276,7 +300,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -284,44 +308,17 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </top>
-      <bottom style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </right>
-      <top style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </top>
-      <bottom style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -656,473 +653,473 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C61D4057-0B41-4F49-BC38-C45ADACA9C0C}">
-  <dimension ref="A1:C63"/>
+  <dimension ref="A1:C70"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.7265625" style="3"/>
-    <col min="3" max="3" width="11.90625" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.7265625" style="2"/>
+    <col min="3" max="3" width="11.90625" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="2">
         <v>648</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" s="2">
         <v>615</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="2">
         <v>612</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5" s="2">
         <v>506</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="2">
         <v>495</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7" s="2">
         <v>436</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="2" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="4">
+      <c r="B8" s="2">
         <v>388</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="2" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="4">
+      <c r="B9" s="2">
         <v>375</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="2" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="4">
+      <c r="B10" s="2">
         <v>314</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="2" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="4">
+      <c r="B11" s="2">
         <v>186</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="2" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="4">
+      <c r="B12" s="2">
         <v>159</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="2" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="4">
+      <c r="B13" s="2">
         <v>126</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="2" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="4">
+      <c r="B14" s="2">
         <v>672</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="2" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="4">
+      <c r="B15" s="2">
         <v>527</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="2" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="4">
+      <c r="B16" s="2">
         <v>474</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="2" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B17" s="4">
+      <c r="B17" s="2">
         <v>437</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="2" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="4">
+      <c r="B18" s="2">
         <v>205</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="2" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="4">
+      <c r="B19" s="2">
         <v>189</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="2" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A20" s="2" t="s">
+      <c r="A20" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B20" s="4">
+      <c r="B20" s="2">
         <v>161</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="2" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A21" s="2" t="s">
+      <c r="A21" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B21" s="4">
+      <c r="B21" s="2">
         <v>67</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="2" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B22" s="4">
+      <c r="B22" s="2">
         <v>55</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C22" s="2" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A23" s="2" t="s">
+      <c r="A23" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B23" s="4">
+      <c r="B23" s="2">
         <v>45</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="2" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A24" s="2" t="s">
+      <c r="A24" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B24" s="4">
+      <c r="B24" s="2">
         <v>553</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C24" s="2" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A25" s="2" t="s">
+      <c r="A25" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B25" s="4">
+      <c r="B25" s="2">
         <v>367</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="C25" s="2" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A26" s="2" t="s">
+      <c r="A26" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B26" s="4">
+      <c r="B26" s="2">
         <v>266</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="2" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A27" s="2" t="s">
+      <c r="A27" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B27" s="4">
+      <c r="B27" s="2">
         <v>259</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C27" s="2" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A28" s="2" t="s">
+      <c r="A28" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B28" s="4">
+      <c r="B28" s="2">
         <v>193</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="C28" s="2" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A29" s="2" t="s">
+      <c r="A29" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B29" s="4">
+      <c r="B29" s="2">
         <v>167</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="C29" s="2" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A30" s="2" t="s">
+      <c r="A30" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B30" s="4">
+      <c r="B30" s="2">
         <v>115</v>
       </c>
-      <c r="C30" s="3" t="s">
+      <c r="C30" s="2" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A31" s="2" t="s">
+      <c r="A31" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B31" s="4">
+      <c r="B31" s="2">
         <v>86</v>
       </c>
-      <c r="C31" s="3" t="s">
+      <c r="C31" s="2" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A32" s="2" t="s">
+      <c r="A32" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B32" s="4">
+      <c r="B32" s="2">
         <v>504</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="C32" s="2" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A33" s="2" t="s">
+      <c r="A33" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B33" s="4">
+      <c r="B33" s="2">
         <v>281</v>
       </c>
-      <c r="C33" s="3" t="s">
+      <c r="C33" s="2" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A34" s="2" t="s">
+      <c r="A34" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B34" s="4">
+      <c r="B34" s="2">
         <v>279</v>
       </c>
-      <c r="C34" s="3" t="s">
+      <c r="C34" s="2" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A35" s="2" t="s">
+      <c r="A35" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B35" s="4">
+      <c r="B35" s="2">
         <v>225</v>
       </c>
-      <c r="C35" s="3" t="s">
+      <c r="C35" s="2" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A36" s="2" t="s">
+      <c r="A36" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B36" s="4">
+      <c r="B36" s="2">
         <v>223</v>
       </c>
-      <c r="C36" s="3" t="s">
+      <c r="C36" s="2" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A37" s="2" t="s">
+      <c r="A37" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B37" s="4">
+      <c r="B37" s="2">
         <v>186</v>
       </c>
-      <c r="C37" s="3" t="s">
+      <c r="C37" s="2" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A38" s="2" t="s">
+      <c r="A38" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B38" s="4">
+      <c r="B38" s="2">
         <v>182</v>
       </c>
-      <c r="C38" s="3" t="s">
+      <c r="C38" s="2" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A39" s="2" t="s">
+      <c r="A39" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B39" s="4">
+      <c r="B39" s="2">
         <v>181</v>
       </c>
-      <c r="C39" s="3" t="s">
+      <c r="C39" s="2" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A40" s="2" t="s">
+      <c r="A40" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B40" s="4">
+      <c r="B40" s="2">
         <v>154</v>
       </c>
-      <c r="C40" s="3" t="s">
+      <c r="C40" s="2" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A41" s="2" t="s">
+      <c r="A41" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B41" s="4">
+      <c r="B41" s="2">
         <v>104</v>
       </c>
-      <c r="C41" s="3" t="s">
+      <c r="C41" s="2" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A42" s="2" t="s">
+      <c r="A42" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B42" s="4">
+      <c r="B42" s="2">
         <v>58</v>
       </c>
-      <c r="C42" s="3" t="s">
+      <c r="C42" s="2" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1130,10 +1127,10 @@
       <c r="A43" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B43" s="3">
+      <c r="B43" s="2">
         <v>305</v>
       </c>
-      <c r="C43" s="3" t="s">
+      <c r="C43" s="2" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1141,10 +1138,10 @@
       <c r="A44" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B44" s="3">
+      <c r="B44" s="2">
         <v>288</v>
       </c>
-      <c r="C44" s="3" t="s">
+      <c r="C44" s="2" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1152,10 +1149,10 @@
       <c r="A45" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B45" s="3">
+      <c r="B45" s="2">
         <v>250</v>
       </c>
-      <c r="C45" s="3" t="s">
+      <c r="C45" s="2" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1163,10 +1160,10 @@
       <c r="A46" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B46" s="3">
+      <c r="B46" s="2">
         <v>211</v>
       </c>
-      <c r="C46" s="3" t="s">
+      <c r="C46" s="2" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1174,10 +1171,10 @@
       <c r="A47" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B47" s="3">
+      <c r="B47" s="2">
         <v>117</v>
       </c>
-      <c r="C47" s="3" t="s">
+      <c r="C47" s="2" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1185,10 +1182,10 @@
       <c r="A48" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B48" s="3">
+      <c r="B48" s="2">
         <v>381</v>
       </c>
-      <c r="C48" s="3" t="s">
+      <c r="C48" s="2" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1196,10 +1193,10 @@
       <c r="A49" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B49" s="3">
+      <c r="B49" s="2">
         <v>275</v>
       </c>
-      <c r="C49" s="3" t="s">
+      <c r="C49" s="2" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1207,10 +1204,10 @@
       <c r="A50" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B50" s="3">
+      <c r="B50" s="2">
         <v>235</v>
       </c>
-      <c r="C50" s="3" t="s">
+      <c r="C50" s="2" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1218,10 +1215,10 @@
       <c r="A51" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B51" s="3">
+      <c r="B51" s="2">
         <v>189</v>
       </c>
-      <c r="C51" s="3" t="s">
+      <c r="C51" s="2" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1229,10 +1226,10 @@
       <c r="A52" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B52" s="3">
+      <c r="B52" s="2">
         <v>172</v>
       </c>
-      <c r="C52" s="3" t="s">
+      <c r="C52" s="2" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1240,10 +1237,10 @@
       <c r="A53" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B53" s="3">
+      <c r="B53" s="2">
         <v>160</v>
       </c>
-      <c r="C53" s="3" t="s">
+      <c r="C53" s="2" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1251,10 +1248,10 @@
       <c r="A54" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B54" s="3">
+      <c r="B54" s="2">
         <v>160</v>
       </c>
-      <c r="C54" s="3" t="s">
+      <c r="C54" s="2" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1262,10 +1259,10 @@
       <c r="A55" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B55" s="3">
+      <c r="B55" s="2">
         <v>154</v>
       </c>
-      <c r="C55" s="3" t="s">
+      <c r="C55" s="2" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1273,10 +1270,10 @@
       <c r="A56" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B56" s="3">
+      <c r="B56" s="2">
         <v>115</v>
       </c>
-      <c r="C56" s="3" t="s">
+      <c r="C56" s="2" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1284,10 +1281,10 @@
       <c r="A57" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="B57" s="3">
+      <c r="B57" s="2">
         <v>107</v>
       </c>
-      <c r="C57" s="3" t="s">
+      <c r="C57" s="2" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1295,10 +1292,10 @@
       <c r="A58" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B58" s="3">
+      <c r="B58" s="2">
         <v>88</v>
       </c>
-      <c r="C58" s="3" t="s">
+      <c r="C58" s="2" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1306,10 +1303,10 @@
       <c r="A59" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="B59" s="3">
+      <c r="B59" s="2">
         <v>264</v>
       </c>
-      <c r="C59" s="3" t="s">
+      <c r="C59" s="2" t="s">
         <v>71</v>
       </c>
     </row>
@@ -1317,10 +1314,10 @@
       <c r="A60" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B60" s="3">
+      <c r="B60" s="2">
         <v>239</v>
       </c>
-      <c r="C60" s="3" t="s">
+      <c r="C60" s="2" t="s">
         <v>71</v>
       </c>
     </row>
@@ -1328,10 +1325,10 @@
       <c r="A61" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B61" s="3">
+      <c r="B61" s="2">
         <v>157</v>
       </c>
-      <c r="C61" s="3" t="s">
+      <c r="C61" s="2" t="s">
         <v>71</v>
       </c>
     </row>
@@ -1339,10 +1336,10 @@
       <c r="A62" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B62" s="3">
+      <c r="B62" s="2">
         <v>142</v>
       </c>
-      <c r="C62" s="3" t="s">
+      <c r="C62" s="2" t="s">
         <v>71</v>
       </c>
     </row>
@@ -1350,11 +1347,88 @@
       <c r="A63" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B63" s="3">
+      <c r="B63" s="2">
         <v>80</v>
       </c>
-      <c r="C63" s="3" t="s">
+      <c r="C63" s="2" t="s">
         <v>71</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A64" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B64" s="3">
+        <v>254</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A65" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B65" s="3">
+        <v>187</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A66" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B66" s="3">
+        <v>113</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A67" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B67" s="3">
+        <v>96</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A68" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B68" s="3">
+        <v>91</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A69" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B69" s="3">
+        <v>62</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A70" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B70" s="3">
+        <v>58</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>